<commit_message>
Fill in net weights from BOS supplier declaration (P. Studecka, 10.07.2026)
- Passschraube 0.0180 kg/pc x 13,000 = 234.00 kg net
- ZB Traeger geschweisst 0.6410 kg/pc x 6,468 = 4,145.99 kg net
- Tare check confirms PL gross 4,862 kg is correct; BL 4,470 kg implausible
- Note: declaration covers weights only, not preferential origin

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kJVMCWg975RAqj8UsDM1d
</commit_message>
<xml_diff>
--- a/output/HS_Code_TARIC_Comparison_BOS_0000462754.xlsx
+++ b/output/HS_Code_TARIC_Comparison_BOS_0000462754.xlsx
@@ -123,10 +123,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -529,7 +529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Zdroj: Sea Waybill KTSATM26006461 (01/06/2026), faktury 0004308261 + 0004308262 (18/03/2026), balicí list 0000462754. Původ: Mexiko (Multitech, Silao). TARIC ověřen k 08/07/2026.</t>
+          <t>Zdroj: Sea Waybill KTSATM26006461 (01/06/2026), faktury 0004308261 + 0004308262 (18/03/2026), balicí list 0000462754, prohlášení dodavatele o čistých váhách BOS/P. Studecká (10/07/2026). Původ: Mexiko (Multitech, Silao). TARIC ověřen k 08/07/2026.</t>
         </is>
       </c>
     </row>
@@ -623,16 +623,14 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Fitted Screw / Tornillo de acero de uso exclusivo automotriz (lícovaný šroub; CZ popis v dokladech není)</t>
+          <t>Fitted Screw / Passschraube / Tornillo de acero de uso exclusivo automotriz (lícovaný šroub; CZ popis v dokladech není)</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
         <v>13000</v>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>CHYBÍ v dokladech</t>
-        </is>
+      <c r="G5" s="6" t="n">
+        <v>234</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>242</v>
@@ -684,16 +682,14 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Traeger Assembly, Audi Q5 / Componente metalico – parte de estructura interna de descansabrazos para automóvil (kovový nosič loketní opěrky; CZ popis v dokladech není)</t>
+          <t>Traeger Assembly, Audi Q5 / ZB Träger geschweisst / Componente metalico – parte de estructura interna de descansabrazos para automóvil (svařovaný kovový nosič loketní opěrky; CZ popis v dokladech není)</t>
         </is>
       </c>
       <c r="F6" s="4" t="n">
         <v>6468</v>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>CHYBÍ v dokladech</t>
-        </is>
+      <c r="G6" s="6" t="n">
+        <v>4145.99</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>4620</v>
@@ -735,7 +731,9 @@
       <c r="F7" s="7" t="n">
         <v>19468</v>
       </c>
-      <c r="G7" s="7" t="n"/>
+      <c r="G7" s="7" t="n">
+        <v>4379.99</v>
+      </c>
       <c r="H7" s="7" t="n">
         <v>4862</v>
       </c>
@@ -764,14 +762,14 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>ČISTÁ HMOTNOST není v žádném dokladu uvedena (jen hrubé hmotnosti na skidech) — sloupec ponechán, hodnoty nutno doplnit od dodavatele.</t>
+          <t>ČISTÉ HMOTNOSTI doplněny dle prohlášení dodavatele (BOS, Petra Studecká, 10.07.2026): Passschraube 0,0180 kg/ks × 13 000 = 234,00 kg; ZB Träger geschweisst 0,6410 kg/ks × 6 468 = 4 145,99 kg. Netto celkem 4 379,99 kg. POZOR: toto prohlášení řeší jen váhy — NENÍ to dodavatelské prohlášení o (preferenčním) původu.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>NESROVNALOSTI V DOKLADECH: BL uvádí 31 skidů / 4 470 kg brutto, balicí list 35 skidů (33× Träger po 140 kg + skidy 34–35 šrouby) / 4 862 kg brutto; skid 35 má v PL hmotnost 0 kg. Před podáním celního prohlášení doporučuji odsouhlasit s dopravcem.</t>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>NESROVNALOSTI V DOKLADECH: BL uvádí 31 skidů / 4 470 kg brutto, balicí list 35 skidů (33× Träger po 140 kg + skidy 34–35 šrouby) / 4 862 kg brutto; skid 35 má v PL hmotnost 0 kg. Kontrola proti nettu 4 379,99 kg: tára u BL by činila jen ~90 kg na 35 skidů (nereálné), u PL ~482 kg (realistické) → správná brutto váha je zjevně 4 862 kg dle PL; BL váhu nechat opravit/vysvětlit dopravcem.</t>
         </is>
       </c>
     </row>
@@ -783,7 +781,7 @@
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Kód 7318 15 95 je doporučená volba pro lícovaný šroub s hlavou jinou než drážkovou/imbus/šestihrannou. Pokud má šroub jiný typ hlavy, viz list 'Alternativy 7318 15' — sazba cla je u všech variant stejná (3,7 %), volba podpoložky tedy nemění výši cla.</t>
         </is>
@@ -1128,7 +1126,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Pozn.: K finálnímu určení stačí od dodavatele zjistit typ hlavy šroubu (výkres položky 990800747702). Sazba cla se volbou podpoložky nemění, ale správný kód je povinný pro celní prohlášení. Samořezné šrouby by patřily do 7318 14, vruty do dřeva 7318 12 — dle popisu 'fitted screw' (lícovaný šroub) jde o strojní šroub → 7318 15.</t>
+          <t>Pozn.: Prohlášení dodavatele (10.07.2026) potvrzuje, že jde o 'Passschraube' (lícovaný šroub). Typické provedení: DIN 609/610 = šestihranná hlava → 7318 15 82 (&lt; 800 MPa) nebo 7318 15 88 (≥ 800 MPa, např. pevnost 8.8/10.9); provedení s válcovou hlavou a imbusem (ISO 7379) → 7318 15 68; jiná hlava → 7318 15 95. K finálnímu určení stačí od dodavatele zjistit typ hlavy a pevnostní třídu (výkres položky 990800747702). Sazba cla se volbou podpoložky nemění (vždy 3,7 %), ale správný kód je povinný pro celní prohlášení. Samořezné šrouby by patřily do 7318 14, vruty do dřeva 7318 12 — Passschraube je strojní šroub → 7318 15.</t>
         </is>
       </c>
     </row>

</xml_diff>